<commit_message>
add 3 YOLO models
</commit_message>
<xml_diff>
--- a/vehicle_counts.xlsx
+++ b/vehicle_counts.xlsx
@@ -490,11 +490,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -515,11 +515,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>motorcycle</t>
+          <t>car</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -540,11 +540,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>truck</t>
+          <t>motorcycle</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -560,16 +560,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -617,15 +617,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:03</t>
+          <t>2026-03-17 16:56:17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -637,11 +637,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:05</t>
+          <t>2026-03-17 16:56:18</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:07</t>
+          <t>2026-03-17 16:56:20</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -677,11 +677,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:09</t>
+          <t>2026-03-17 16:56:22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -697,15 +697,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:10</t>
+          <t>2026-03-17 16:56:23</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>motorcycle</t>
+          <t>car</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -717,15 +717,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:11</t>
+          <t>2026-03-17 16:56:25</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -737,15 +737,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:15</t>
+          <t>2026-03-17 16:56:26</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>37</v>
+        <v>120</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>motorcycle</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -757,15 +757,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:17</t>
+          <t>2026-03-17 16:56:27</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>truck</t>
+          <t>motorcycle</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -777,11 +777,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:18</t>
+          <t>2026-03-17 16:56:29</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -797,15 +797,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:20</t>
+          <t>2026-03-17 16:56:31</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>truck</t>
+          <t>car</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -817,11 +817,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:23</t>
+          <t>2026-03-17 16:56:33</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -837,15 +837,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:26</t>
+          <t>2026-03-17 16:56:35</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>179</v>
+        <v>145</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -857,15 +857,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:29</t>
+          <t>2026-03-17 16:56:37</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>190</v>
+        <v>227</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -877,11 +877,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:33</t>
+          <t>2026-03-17 16:56:39</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>271</v>
+        <v>197</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -897,11 +897,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:34</t>
+          <t>2026-03-17 16:56:41</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>293</v>
+        <v>212</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -917,15 +917,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:36</t>
+          <t>2026-03-17 16:56:41</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>311</v>
+        <v>263</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>truck</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -937,11 +937,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:38</t>
+          <t>2026-03-17 16:56:42</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>285</v>
+        <v>220</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -957,15 +957,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-17 16:38:39</t>
+          <t>2026-03-17 16:56:45</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>car</t>
+          <t>motorcycle</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -977,11 +977,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-17 16:39:23</t>
+          <t>2026-03-17 16:56:46</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>414</v>
+        <v>308</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -990,18 +990,18 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-17 16:39:24</t>
+          <t>2026-03-17 16:56:49</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>416</v>
+        <v>274</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1009,6 +1009,926 @@
         </is>
       </c>
       <c r="D21" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:56:49</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>275</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:56:52</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>362</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:56:55</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>332</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:56:58</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>336</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:56:58</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>316</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:01</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>394</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:03</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>461</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:05</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>437</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:06</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>453</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:09</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>423</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:12</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>493</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:15</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>499</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:17</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>580</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:19</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>562</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:20</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>596</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:24</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>606</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:26</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>601</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:33</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>698</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:36</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>736</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:40</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>727</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:44</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>810</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>motorcycle</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:47</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>862</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>motorcycle</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:47</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>991</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>motorcycle</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:49</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1046</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:52</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:52</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1049</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:52</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1074</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:55</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:56</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:56</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1178</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:58</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:57:59</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1152</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:00</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1199</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:01</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1135</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:02</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1257</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:04</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1289</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:05</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1327</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:05</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1409</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:08</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1438</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:08</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:13</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1587</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:15</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1608</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:16</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1560</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>truck</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:16</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1612</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:16</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1662</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Inbound</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-17 16:58:18</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1583</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>car</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>Inbound</t>
         </is>

</xml_diff>